<commit_message>
Added a few more traits.
</commit_message>
<xml_diff>
--- a/story_simulator/data/character_quirks.xlsx
+++ b/story_simulator/data/character_quirks.xlsx
@@ -5,7 +5,7 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/zhafen/repos/stories/allsides/world/characters/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/zhafen/repos/story-simulator/story_simulator/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="33" uniqueCount="33">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="43" uniqueCount="43">
   <si>
     <t>Description</t>
   </si>
@@ -126,6 +126,36 @@
   </si>
   <si>
     <t>Carries around a plant as a pet/has a plant growing out of them</t>
+  </si>
+  <si>
+    <t>Scared of the supernatural</t>
+  </si>
+  <si>
+    <t>Hates things of a certain shape</t>
+  </si>
+  <si>
+    <t>Sits weirdly</t>
+  </si>
+  <si>
+    <t>Makes up slang</t>
+  </si>
+  <si>
+    <t>Makes exaggerated gestures (e.g. double thumbs up)</t>
+  </si>
+  <si>
+    <t>Thinks out loud</t>
+  </si>
+  <si>
+    <t>Stops/starts in the middle of a sentence</t>
+  </si>
+  <si>
+    <t>Often walks weirdly (e.g. skips/marches/etc)</t>
+  </si>
+  <si>
+    <t>Changes their attire frequently</t>
+  </si>
+  <si>
+    <t>Usually looking for a snack</t>
   </si>
 </sst>
 </file>
@@ -446,7 +476,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:C32"/>
+  <dimension ref="A1:C42"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="12.33203125" customWidth="1"/>
@@ -712,6 +742,83 @@
         <v>32</v>
       </c>
     </row>
+    <row r="33" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A33">
+        <v>1</v>
+      </c>
+      <c r="B33" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="34" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A34">
+        <v>1</v>
+      </c>
+      <c r="B34" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="35" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A35">
+        <v>1</v>
+      </c>
+      <c r="B35" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="36" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A36">
+        <v>1</v>
+      </c>
+      <c r="B36" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="37" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A37">
+        <v>1</v>
+      </c>
+      <c r="B37" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="38" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A38">
+        <v>1</v>
+      </c>
+      <c r="B38" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="39" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A39">
+        <v>1</v>
+      </c>
+      <c r="B39" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="40" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A40">
+        <v>1</v>
+      </c>
+      <c r="B40" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="41" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A41">
+        <v>1</v>
+      </c>
+      <c r="B41" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="42" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="B42" t="s">
+        <v>42</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Finished putting in character trait data.
</commit_message>
<xml_diff>
--- a/story_simulator/data/character_quirks.xlsx
+++ b/story_simulator/data/character_quirks.xlsx
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="43" uniqueCount="43">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="44" uniqueCount="44">
   <si>
     <t>Description</t>
   </si>
@@ -156,6 +156,9 @@
   </si>
   <si>
     <t>Usually looking for a snack</t>
+  </si>
+  <si>
+    <t>Dresses in formal wear/rags</t>
   </si>
 </sst>
 </file>
@@ -476,7 +479,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:C42"/>
+  <dimension ref="A1:C43"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="12.33203125" customWidth="1"/>
@@ -819,6 +822,11 @@
         <v>42</v>
       </c>
     </row>
+    <row r="43" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="B43" t="s">
+        <v>43</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Added more character quirks.
</commit_message>
<xml_diff>
--- a/story_simulator/data/character_quirks.xlsx
+++ b/story_simulator/data/character_quirks.xlsx
@@ -9,7 +9,7 @@
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
-    <workbookView xWindow="0" yWindow="460" windowWidth="25600" windowHeight="14100" tabRatio="500"/>
+    <workbookView xWindow="860" yWindow="460" windowWidth="25600" windowHeight="14100" tabRatio="500"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="44" uniqueCount="44">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="70" uniqueCount="70">
   <si>
     <t>Description</t>
   </si>
@@ -119,9 +119,6 @@
     <t>Embarrassed easily/rarily</t>
   </si>
   <si>
-    <t>Forgetful/has a good memory</t>
-  </si>
-  <si>
     <t>Hates walking</t>
   </si>
   <si>
@@ -159,13 +156,94 @@
   </si>
   <si>
     <t>Dresses in formal wear/rags</t>
+  </si>
+  <si>
+    <t>Uses jargon</t>
+  </si>
+  <si>
+    <t>Subject to malapropisms/mispronounces</t>
+  </si>
+  <si>
+    <t>Ends sentences as a question (interrogative inflection)</t>
+  </si>
+  <si>
+    <t>Smiles when unsure</t>
+  </si>
+  <si>
+    <t>Rarely smiles/always smiles</t>
+  </si>
+  <si>
+    <t>Cries easily</t>
+  </si>
+  <si>
+    <t>Directs conversation, only listens to the other person when it suits them</t>
+  </si>
+  <si>
+    <t>Uses self-deprecation as a humor device</t>
+  </si>
+  <si>
+    <t>Mimics others sarcastically</t>
+  </si>
+  <si>
+    <t>Sighs frequently</t>
+  </si>
+  <si>
+    <t>Gets humor out of making others/friends uncomfortable</t>
+  </si>
+  <si>
+    <t>Makes exaggerated sounds when they're lightly upset (hisses, "awawawa")</t>
+  </si>
+  <si>
+    <t>Uses a pleading voice regularly/semi-regularly</t>
+  </si>
+  <si>
+    <t>Doesn't eat all their food/wipes their plate clean</t>
+  </si>
+  <si>
+    <t>Always collecting things</t>
+  </si>
+  <si>
+    <t>Goes through self-improvement phases</t>
+  </si>
+  <si>
+    <t>Goes through hobbies/obsessions</t>
+  </si>
+  <si>
+    <t>Carries something they fiddle with (e.g. a coin/stick/rope)</t>
+  </si>
+  <si>
+    <t>Always trying to learn a new trick (e.g. cards/juggling)</t>
+  </si>
+  <si>
+    <t>Always doing something with their hands (e.g. knitting/breaking things apart)</t>
+  </si>
+  <si>
+    <t>Hesitates before responding</t>
+  </si>
+  <si>
+    <t>Tries to learn new lingo</t>
+  </si>
+  <si>
+    <t>Only speaks when they're very confident</t>
+  </si>
+  <si>
+    <t>Shrugs/gestures frequently</t>
+  </si>
+  <si>
+    <t>Always takes notes</t>
+  </si>
+  <si>
+    <t>Pushes conversations towards being very long/brief</t>
+  </si>
+  <si>
+    <t>Great/terrible with names</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -177,6 +255,12 @@
       <sz val="11"/>
       <color rgb="FF000000"/>
       <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="12"/>
+      <color rgb="FF333333"/>
+      <name val="Calibri"/>
+      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="2">
@@ -199,9 +283,10 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -479,11 +564,11 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:C43"/>
+  <dimension ref="A1:C69"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="12.33203125" customWidth="1"/>
-    <col min="2" max="2" width="57.5" customWidth="1"/>
+    <col min="2" max="2" width="61" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.2">
@@ -723,7 +808,7 @@
     </row>
     <row r="30" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A30">
-        <v>0.5</v>
+        <v>1</v>
       </c>
       <c r="B30" t="s">
         <v>30</v>
@@ -818,13 +903,227 @@
       </c>
     </row>
     <row r="42" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A42">
+        <v>1</v>
+      </c>
       <c r="B42" t="s">
         <v>42</v>
       </c>
     </row>
     <row r="43" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="B43" t="s">
+      <c r="A43">
+        <v>1</v>
+      </c>
+      <c r="B43" s="2" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="44" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A44">
+        <v>1</v>
+      </c>
+      <c r="B44" t="s">
         <v>43</v>
+      </c>
+    </row>
+    <row r="45" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A45">
+        <v>1</v>
+      </c>
+      <c r="B45" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="46" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A46">
+        <v>1</v>
+      </c>
+      <c r="B46" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="47" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A47">
+        <v>1</v>
+      </c>
+      <c r="B47" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="48" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A48">
+        <v>1</v>
+      </c>
+      <c r="B48" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="49" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A49">
+        <v>1</v>
+      </c>
+      <c r="B49" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="50" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A50">
+        <v>1</v>
+      </c>
+      <c r="B50" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="51" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A51">
+        <v>1</v>
+      </c>
+      <c r="B51" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="52" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A52">
+        <v>1</v>
+      </c>
+      <c r="B52" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="53" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A53">
+        <v>1</v>
+      </c>
+      <c r="B53" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="54" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A54">
+        <v>1</v>
+      </c>
+      <c r="B54" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="55" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A55">
+        <v>1</v>
+      </c>
+      <c r="B55" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="56" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A56">
+        <v>1</v>
+      </c>
+      <c r="B56" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="57" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A57">
+        <v>1</v>
+      </c>
+      <c r="B57" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="58" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A58">
+        <v>1</v>
+      </c>
+      <c r="B58" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="59" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A59">
+        <v>1</v>
+      </c>
+      <c r="B59" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="60" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A60">
+        <v>1</v>
+      </c>
+      <c r="B60" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="61" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A61">
+        <v>1</v>
+      </c>
+      <c r="B61" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="62" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A62">
+        <v>1</v>
+      </c>
+      <c r="B62" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="63" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A63">
+        <v>1</v>
+      </c>
+      <c r="B63" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="64" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A64">
+        <v>1</v>
+      </c>
+      <c r="B64" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="65" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A65">
+        <v>1</v>
+      </c>
+      <c r="B65" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="66" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A66">
+        <v>1</v>
+      </c>
+      <c r="B66" t="s">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="67" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A67">
+        <v>1</v>
+      </c>
+      <c r="B67" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="68" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A68">
+        <v>1</v>
+      </c>
+      <c r="B68" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="69" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A69">
+        <v>1</v>
+      </c>
+      <c r="B69" t="s">
+        <v>69</v>
       </c>
     </row>
   </sheetData>

</xml_diff>